<commit_message>
Review fixes: area left to the appraiser, recorded sale first, meaning check scope, row and type checks, grantor and grantee
</commit_message>
<xml_diff>
--- a/site/dist/files/comparable-1-entered.xlsx
+++ b/site/dist/files/comparable-1-entered.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="55">
   <si>
     <t>Sales comparison grid (demonstration template)</t>
   </si>
   <si>
-    <t>Blue cells: reported facts, entered from approved records. Yellow cells: appraiser input. A blank adjustment is not zero: adjusted lines stay blank until the adjustments above them are entered.</t>
+    <t>Blue cells: reported facts, entered from approved records. Yellow cells: appraiser input, including the building area used for comparison. A blank input is not zero: calculated lines stay blank until their inputs are filled.</t>
   </si>
   <si>
     <t>Subject</t>
@@ -49,13 +49,16 @@
     <t>Recorded instrument</t>
   </si>
   <si>
-    <t>Sale date</t>
+    <t>Sale date (county record)</t>
   </si>
   <si>
     <t>Sale price ($)</t>
   </si>
   <si>
-    <t>Gross building area (sq ft, above grade)</t>
+    <t>Building area for comparison (sq ft), appraiser's choice</t>
+  </si>
+  <si>
+    <t>Building area as reported by each source</t>
   </si>
   <si>
     <t>Land area (acres)</t>
@@ -67,10 +70,22 @@
     <t>Zoning</t>
   </si>
   <si>
-    <t>Property rights conveyed (reported)</t>
-  </si>
-  <si>
-    <t>Conditions of sale (reported facts)</t>
+    <t>Grantor (seller)</t>
+  </si>
+  <si>
+    <t>Grantee (buyer)</t>
+  </si>
+  <si>
+    <t>Property rights (reported)</t>
+  </si>
+  <si>
+    <t>Conditions of sale (reported)</t>
+  </si>
+  <si>
+    <t>Marketing history (reported)</t>
+  </si>
+  <si>
+    <t>Non-realty items (reported)</t>
   </si>
   <si>
     <t>Sources</t>
@@ -79,10 +94,10 @@
     <t>Verification</t>
   </si>
   <si>
-    <t>Calculated from reported facts</t>
-  </si>
-  <si>
-    <t>Sale price per sq ft of gross building area</t>
+    <t>Calculated from reported facts and the chosen area</t>
+  </si>
+  <si>
+    <t>Sale price per sq ft of the chosen building area</t>
   </si>
   <si>
     <t>Land-to-building ratio</t>
@@ -308,15 +323,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFE2D3A8"/>
       </left>
@@ -331,11 +337,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -361,13 +376,16 @@
     <xf numFmtId="165" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="166" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -376,13 +394,13 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -397,7 +415,7 @@
     <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -705,11 +723,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B2:F50"/>
+  <dimension ref="B2:F55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.7109375" customWidth="1"/>
-    <col min="2" max="2" width="38.7109375" customWidth="1"/>
+    <col min="2" max="2" width="40.7109375" customWidth="1"/>
     <col min="3" max="6" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -803,23 +821,23 @@
       <c r="B10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8">
-        <v>7354.0</v>
-      </c>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9">
-        <v>0.57</v>
-      </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>County assessor: 7,354 sq ft on floor lines 1 to 3, plus 2,644 on lower-level lines B1. Listing site: 6,000 sq ft. MLS: 2 stories.</t>
+        </is>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" spans="2:6">
       <c r="B12" s="4" t="s">
@@ -827,7 +845,7 @@
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10">
-        <v>1890.0</v>
+        <v>0.57</v>
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -836,25 +854,23 @@
       <c r="B13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="C13" s="11"/>
+      <c r="D13" s="11">
+        <v>1890.0</v>
+      </c>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+    </row>
+    <row r="14" spans="2:6">
+      <c r="B14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>BC and R-6</t>
         </is>
       </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-    </row>
-    <row r="14" spans="2:6">
-      <c r="B14" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Fee Simple (reported by MLS)</t>
-        </is>
-      </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
     </row>
@@ -865,7 +881,7 @@
       <c r="C15" s="6"/>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Offer accepted by the borough council with no contingencies and closing in 30 days or as soon as possible (minutes of 9/11/2025). Listed at $575,000 on 1/10/2025, reduced to $499,000 on 7/15/2025. Excluded: furniture, fixtures, equipment and inventory of seller.</t>
+          <t>St. Lawrence Borough; the property is the former borough hall</t>
         </is>
       </c>
       <c r="E15" s="5"/>
@@ -875,431 +891,505 @@
       <c r="B16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="5"/>
+      <c r="C16" s="6"/>
       <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Molnar Holdings LLC (current owner per county record, not read from the deed)</t>
+        </is>
+      </c>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+    </row>
+    <row r="17" spans="2:6">
+      <c r="B17" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="6"/>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Fee Simple, per the MLS Ownership field; not verified</t>
+        </is>
+      </c>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="2:6">
+      <c r="B18" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="6"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>No contingencies; closing in 30 days or as soon as possible (council motion, 9/11/2025)</t>
+        </is>
+      </c>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="6"/>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Listed at $575,000 on 1/10/2025; reduced to $499,000 on 7/15/2025; sold on 10/10/2025 (MLS history)</t>
+        </is>
+      </c>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="B20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Excluded from the sale: furniture, fixtures, equipment and inventory of seller (MLS)</t>
+        </is>
+      </c>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" spans="2:6">
+      <c r="B21" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Berks County assessment record (open data, retrieved 9/30/2026); St. Lawrence Borough Council minutes, 9/11/2025; MLS PABK2052516 on two listing sites</t>
         </is>
       </c>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-    </row>
-    <row r="17" spans="2:6">
-      <c r="B17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" spans="2:6">
+      <c r="B22" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Public records reviewed; no transaction-party verification performed</t>
         </is>
       </c>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="19" spans="2:6">
-      <c r="B19" s="11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6">
-      <c r="B20" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D20" s="12">
-        <f>IF(OR(D9="",D10=""),"",D9/D10)</f>
-        <v/>
-      </c>
-      <c r="E20" s="12">
-        <f>IF(OR(E9="",E10=""),"",E9/E10)</f>
-        <v/>
-      </c>
-      <c r="F20" s="12">
-        <f>IF(OR(F9="",F10=""),"",F9/F10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="2:6">
-      <c r="B21" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="13">
-        <f>IF(OR(C11="",C10=""),"",C11*SqFtPerAcre/C10)</f>
-        <v/>
-      </c>
-      <c r="D21" s="13">
-        <f>IF(OR(D11="",D10=""),"",D11*SqFtPerAcre/D10)</f>
-        <v/>
-      </c>
-      <c r="E21" s="13">
-        <f>IF(OR(E11="",E10=""),"",E11*SqFtPerAcre/E10)</f>
-        <v/>
-      </c>
-      <c r="F21" s="13">
-        <f>IF(OR(F11="",F10=""),"",F11*SqFtPerAcre/F10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="2:6">
-      <c r="B22" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6">
-      <c r="B23" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
     </row>
     <row r="24" spans="2:6">
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="12" t="s">
         <v>24</v>
-      </c>
-      <c r="D24" s="12">
-        <f>IF(OR(D20="",D23=""),"",D20*(1+D23))</f>
-        <v/>
-      </c>
-      <c r="E24" s="12">
-        <f>IF(OR(E20="",E23=""),"",E20*(1+E23))</f>
-        <v/>
-      </c>
-      <c r="F24" s="12">
-        <f>IF(OR(F20="",F23=""),"",F20*(1+F23))</f>
-        <v/>
       </c>
     </row>
     <row r="25" spans="2:6">
       <c r="B25" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
+      <c r="D25" s="13">
+        <f>IF(OR(D9="",D10=""),"",D9/D10)</f>
+        <v/>
+      </c>
+      <c r="E25" s="13">
+        <f>IF(OR(E9="",E10=""),"",E9/E10)</f>
+        <v/>
+      </c>
+      <c r="F25" s="13">
+        <f>IF(OR(F9="",F10=""),"",F9/F10)</f>
+        <v/>
+      </c>
     </row>
     <row r="26" spans="2:6">
-      <c r="B26" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D26" s="12">
-        <f>IF(OR(D24="",D25=""),"",D24*(1+D25))</f>
-        <v/>
-      </c>
-      <c r="E26" s="12">
-        <f>IF(OR(E24="",E25=""),"",E24*(1+E25))</f>
-        <v/>
-      </c>
-      <c r="F26" s="12">
-        <f>IF(OR(F24="",F25=""),"",F24*(1+F25))</f>
+      <c r="B26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" s="14">
+        <f>IF(OR(C12="",C10=""),"",C12*SqFtPerAcre/C10)</f>
+        <v/>
+      </c>
+      <c r="D26" s="14">
+        <f>IF(OR(D12="",D10=""),"",D12*SqFtPerAcre/D10)</f>
+        <v/>
+      </c>
+      <c r="E26" s="14">
+        <f>IF(OR(E12="",E10=""),"",E12*SqFtPerAcre/E10)</f>
+        <v/>
+      </c>
+      <c r="F26" s="14">
+        <f>IF(OR(F12="",F10=""),"",F12*SqFtPerAcre/F10)</f>
         <v/>
       </c>
     </row>
     <row r="27" spans="2:6">
-      <c r="B27" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
+      <c r="B27" s="12" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="28" spans="2:6">
-      <c r="B28" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D28" s="12">
-        <f>IF(OR(D26="",D27=""),"",D26*(1+D27))</f>
-        <v/>
-      </c>
-      <c r="E28" s="12">
-        <f>IF(OR(E26="",E27=""),"",E26*(1+E27))</f>
-        <v/>
-      </c>
-      <c r="F28" s="12">
-        <f>IF(OR(F26="",F27=""),"",F26*(1+F27))</f>
-        <v/>
-      </c>
+      <c r="B28" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
     </row>
     <row r="29" spans="2:6">
-      <c r="B29" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
+      <c r="B29" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D29" s="13">
+        <f>IF(OR(D25="",D28=""),"",D25*(1+D28))</f>
+        <v/>
+      </c>
+      <c r="E29" s="13">
+        <f>IF(OR(E25="",E28=""),"",E25*(1+E28))</f>
+        <v/>
+      </c>
+      <c r="F29" s="13">
+        <f>IF(OR(F25="",F28=""),"",F25*(1+F28))</f>
+        <v/>
+      </c>
     </row>
     <row r="30" spans="2:6">
-      <c r="B30" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D30" s="12">
-        <f>IF(OR(D28="",D29=""),"",D28+D29)</f>
-        <v/>
-      </c>
-      <c r="E30" s="12">
-        <f>IF(OR(E28="",E29=""),"",E28+E29)</f>
-        <v/>
-      </c>
-      <c r="F30" s="12">
-        <f>IF(OR(F28="",F29=""),"",F28+F29)</f>
-        <v/>
-      </c>
+      <c r="B30" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
     </row>
     <row r="31" spans="2:6">
-      <c r="B31" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
+      <c r="B31" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D31" s="13">
+        <f>IF(OR(D29="",D30=""),"",D29*(1+D30))</f>
+        <v/>
+      </c>
+      <c r="E31" s="13">
+        <f>IF(OR(E29="",E30=""),"",E29*(1+E30))</f>
+        <v/>
+      </c>
+      <c r="F31" s="13">
+        <f>IF(OR(F29="",F30=""),"",F29*(1+F30))</f>
+        <v/>
+      </c>
     </row>
     <row r="32" spans="2:6">
-      <c r="B32" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D32" s="12">
-        <f>IF(OR(D30="",D31=""),"",D30*(1+D31))</f>
-        <v/>
-      </c>
-      <c r="E32" s="12">
-        <f>IF(OR(E30="",E31=""),"",E30*(1+E31))</f>
-        <v/>
-      </c>
-      <c r="F32" s="12">
-        <f>IF(OR(F30="",F31=""),"",F30*(1+F31))</f>
+      <c r="B32" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+    </row>
+    <row r="33" spans="2:6">
+      <c r="B33" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D33" s="13">
+        <f>IF(OR(D31="",D32=""),"",D31*(1+D32))</f>
+        <v/>
+      </c>
+      <c r="E33" s="13">
+        <f>IF(OR(E31="",E32=""),"",E31*(1+E32))</f>
+        <v/>
+      </c>
+      <c r="F33" s="13">
+        <f>IF(OR(F31="",F32=""),"",F31*(1+F32))</f>
         <v/>
       </c>
     </row>
     <row r="34" spans="2:6">
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+    </row>
+    <row r="35" spans="2:6">
+      <c r="B35" s="16" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="35" spans="2:6">
-      <c r="B35" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
+      <c r="D35" s="13">
+        <f>IF(OR(D33="",D34=""),"",D33+D34)</f>
+        <v/>
+      </c>
+      <c r="E35" s="13">
+        <f>IF(OR(E33="",E34=""),"",E33+E34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="13">
+        <f>IF(OR(F33="",F34=""),"",F33+F34)</f>
+        <v/>
+      </c>
     </row>
     <row r="36" spans="2:6">
       <c r="B36" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
+        <v>33</v>
+      </c>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
     </row>
     <row r="37" spans="2:6">
-      <c r="B37" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-    </row>
-    <row r="38" spans="2:6">
-      <c r="B38" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
+      <c r="B37" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D37" s="13">
+        <f>IF(OR(D35="",D36=""),"",D35*(1+D36))</f>
+        <v/>
+      </c>
+      <c r="E37" s="13">
+        <f>IF(OR(E35="",E36=""),"",E35*(1+E36))</f>
+        <v/>
+      </c>
+      <c r="F37" s="13">
+        <f>IF(OR(F35="",F36=""),"",F35*(1+F36))</f>
+        <v/>
+      </c>
     </row>
     <row r="39" spans="2:6">
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
     </row>
     <row r="40" spans="2:6">
       <c r="B40" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
     </row>
     <row r="41" spans="2:6">
       <c r="B41" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
     </row>
     <row r="42" spans="2:6">
       <c r="B42" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D42" s="17">
-        <f>IF(COUNTBLANK(D35:D41)&gt;0,"",SUM(D35:D41))</f>
-        <v/>
-      </c>
-      <c r="E42" s="17">
-        <f>IF(COUNTBLANK(E35:E41)&gt;0,"",SUM(E35:E41))</f>
-        <v/>
-      </c>
-      <c r="F42" s="17">
-        <f>IF(COUNTBLANK(F35:F41)&gt;0,"",SUM(F35:F41))</f>
-        <v/>
-      </c>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
     </row>
     <row r="43" spans="2:6">
-      <c r="B43" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="D43" s="19">
-        <f>IF(OR(D32="",D42=""),"",D32*(1+D42))</f>
-        <v/>
-      </c>
-      <c r="E43" s="19">
-        <f>IF(OR(E32="",E42=""),"",E32*(1+E42))</f>
-        <v/>
-      </c>
-      <c r="F43" s="19">
-        <f>IF(OR(F32="",F42=""),"",F32*(1+F42))</f>
-        <v/>
-      </c>
+      <c r="B43" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
     </row>
     <row r="44" spans="2:6">
       <c r="B44" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D44" s="17">
-        <f>IF(D43="","",(ABS(D23)*D20+ABS(D25)*D24+ABS(D27)*D26+ABS(D29)+ABS(D31)*D30+SUMPRODUCT(ABS(D35:D41))*D32)/D20)</f>
-        <v>0</v>
-      </c>
-      <c r="E44" s="17">
-        <f>IF(E43="","",(ABS(E23)*E20+ABS(E25)*E24+ABS(E27)*E26+ABS(E29)+ABS(E31)*E30+SUMPRODUCT(ABS(E35:E41))*E32)/E20)</f>
-        <v>0</v>
-      </c>
-      <c r="F44" s="17">
-        <f>IF(F43="","",(ABS(F23)*F20+ABS(F25)*F24+ABS(F27)*F26+ABS(F29)+ABS(F31)*F30+SUMPRODUCT(ABS(F35:F41))*F32)/F20)</f>
-        <v>0</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
     </row>
     <row r="45" spans="2:6">
       <c r="B45" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D45" s="17">
-        <f>IF(D43="","",D43/D20-1)</f>
-        <v/>
-      </c>
-      <c r="E45" s="17">
-        <f>IF(E43="","",E43/E20-1)</f>
-        <v/>
-      </c>
-      <c r="F45" s="17">
-        <f>IF(F43="","",F43/F20-1)</f>
-        <v/>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+    </row>
+    <row r="46" spans="2:6">
+      <c r="B46" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
     </row>
     <row r="47" spans="2:6">
-      <c r="B47" s="11" t="s">
-        <v>40</v>
+      <c r="B47" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D47" s="18">
+        <f>IF(COUNTBLANK(D40:D46)&gt;0,"",SUM(D40:D46))</f>
+        <v/>
+      </c>
+      <c r="E47" s="18">
+        <f>IF(COUNTBLANK(E40:E46)&gt;0,"",SUM(E40:E46))</f>
+        <v/>
+      </c>
+      <c r="F47" s="18">
+        <f>IF(COUNTBLANK(F40:F46)&gt;0,"",SUM(F40:F46))</f>
+        <v/>
       </c>
     </row>
     <row r="48" spans="2:6">
-      <c r="B48" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C48" s="16"/>
-    </row>
-    <row r="49" spans="2:3">
-      <c r="B49" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="C49" s="20">
-        <f>IF(OR(C48="",C10=""),"",ROUND(C48*C10,ValueRounding))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="2:3">
+      <c r="B48" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D48" s="20">
+        <f>IF(OR(D37="",D47=""),"",D37*(1+D47))</f>
+        <v/>
+      </c>
+      <c r="E48" s="20">
+        <f>IF(OR(E37="",E47=""),"",E37*(1+E47))</f>
+        <v/>
+      </c>
+      <c r="F48" s="20">
+        <f>IF(OR(F37="",F47=""),"",F37*(1+F47))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="2:6">
+      <c r="B49" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D49" s="18">
+        <f>IF(D48="","",(ABS(D28)*D25+ABS(D30)*D29+ABS(D32)*D31+ABS(D34)+ABS(D36)*D35+SUMPRODUCT(ABS(D40:D46))*D37)/D25)</f>
+        <v/>
+      </c>
+      <c r="E49" s="18">
+        <f>IF(E48="","",(ABS(E28)*E25+ABS(E30)*E29+ABS(E32)*E31+ABS(E34)+ABS(E36)*E35+SUMPRODUCT(ABS(E40:E46))*E37)/E25)</f>
+        <v/>
+      </c>
+      <c r="F49" s="18">
+        <f>IF(F48="","",(ABS(F28)*F25+ABS(F30)*F29+ABS(F32)*F31+ABS(F34)+ABS(F36)*F35+SUMPRODUCT(ABS(F40:F46))*F37)/F25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="2:6">
       <c r="B50" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C50" s="21"/>
+        <v>44</v>
+      </c>
+      <c r="D50" s="18">
+        <f>IF(D48="","",D48/D25-1)</f>
+        <v/>
+      </c>
+      <c r="E50" s="18">
+        <f>IF(E48="","",E48/E25-1)</f>
+        <v/>
+      </c>
+      <c r="F50" s="18">
+        <f>IF(F48="","",F48/F25-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="2:6">
+      <c r="B52" s="12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6">
+      <c r="B53" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C53" s="17"/>
+    </row>
+    <row r="54" spans="2:6">
+      <c r="B54" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C54" s="21">
+        <f>IF(OR(C53="",C10=""),"",ROUND(C53*C10,ValueRounding))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="2:6">
+      <c r="B55" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C55" s="22"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D44:F44">
+  <conditionalFormatting sqref="D49:F49">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AND(ISNUMBER(D44),D44&gt;GrossAdjustmentFlag)</formula>
+      <formula>AND(ISNUMBER(D49),D49&gt;GrossAdjustmentFlag)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="18">
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="D23">
+  <dataValidations count="21">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="D28">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="D25">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="D30">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="D27">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="D32">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="D31">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="D36">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D35:D41">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D40:D46">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
     <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8">
       <formula1>36526</formula1>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="E23">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Pick the building area basis from the reported areas above" sqref="D10">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="E28">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="E25">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="E30">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="E27">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="E32">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="E31">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="E36">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E35:E41">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E40:E46">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
     <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E8">
       <formula1>36526</formula1>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="F23">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Pick the building area basis from the reported areas above" sqref="E10">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="F28">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="F25">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="F30">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="F27">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="F32">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="F31">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Percentage, for example 5% or -3%" sqref="F36">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F35:F41">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F40:F46">
       <formula1>-0.5</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
     <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F8">
       <formula1>36526</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Appraiser input" prompt="Pick the building area basis from the reported areas above" sqref="F10">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1313,15 +1403,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B2">
         <v>43560</v>
@@ -1329,7 +1419,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B3">
         <v>-3</v>
@@ -1337,7 +1427,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B4">
         <v>0.25</v>
@@ -1345,11 +1435,11 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B6">
-        <f>COUNTA('Sales Comparison'!D5:D17)</f>
-        <v>0</v>
+        <f>COUNTA('Sales Comparison'!D5:D22)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Judge fixes: label and unit binding, three-state resume, array ranges refused, per-document sources, source links and evidence package, generated destination, honest scope
</commit_message>
<xml_diff>
--- a/site/dist/files/comparable-1-entered.xlsx
+++ b/site/dist/files/comparable-1-entered.xlsx
@@ -70,10 +70,10 @@
     <t>Zoning</t>
   </si>
   <si>
-    <t>Grantor (seller)</t>
-  </si>
-  <si>
-    <t>Grantee (buyer)</t>
+    <t>Seller (reported in council minutes)</t>
+  </si>
+  <si>
+    <t>Current owner (county record)</t>
   </si>
   <si>
     <t>Property rights (reported)</t>
@@ -894,7 +894,7 @@
       <c r="C16" s="6"/>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Molnar Holdings LLC (current owner per county record, not read from the deed)</t>
+          <t>Molnar Holdings LLC; buyer not read from the deed</t>
         </is>
       </c>
       <c r="E16" s="5"/>

</xml_diff>